<commit_message>
Tighten Chuangdi quote skills for missing pitch, BOM rollup, and demo costs.
Ask users when tender pitch is absent, recompute aux/pack from BOM when summary cells are empty formulas, and seed readable demo rollups without pricing LEDs into iron-box auxiliaries.
</commit_message>
<xml_diff>
--- a/chuangdi/数据/核算口径表-演示.xlsx
+++ b/chuangdi/数据/核算口径表-演示.xlsx
@@ -489,7 +489,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>【演示副本】已为辅材 BOM 空单价与每平米收口大件单价列填入模拟数（黄底）。正式稿大件单价仍应留空、取自规格单价表。本文件不是创迪成本。</t>
+          <t>【演示副本】已为辅材 BOM 空单价填模拟数，并按公式骨架滚出行合计与 1㎡ 辅料/包材汇总（黄底）。正式稿大件单价仍应留空、取自规格单价表；正式稿汇总格保留公式，须在 Excel 中打开计算或由人维护滚出值。本文件不是创迪成本。</t>
         </is>
       </c>
     </row>
@@ -581,9 +581,8 @@
       <c r="E3" t="n">
         <v>1</v>
       </c>
-      <c r="F3">
-        <f>D3*E3</f>
-        <v/>
+      <c r="F3" s="1" t="n">
+        <v>880</v>
       </c>
     </row>
     <row r="4">
@@ -608,9 +607,8 @@
       <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="F4">
-        <f>D4*E4</f>
-        <v/>
+      <c r="F4" s="1" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -635,9 +633,8 @@
       <c r="E5" t="n">
         <v>1</v>
       </c>
-      <c r="F5">
-        <f>D5*E5</f>
-        <v/>
+      <c r="F5" s="1" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="6">
@@ -675,9 +672,8 @@
       <c r="E9" t="n">
         <v>144</v>
       </c>
-      <c r="F9">
-        <f>D9*E9</f>
-        <v/>
+      <c r="F9" s="1" t="n">
+        <v>17.28</v>
       </c>
     </row>
     <row r="10">
@@ -702,9 +698,8 @@
       <c r="E10" t="n">
         <v>24</v>
       </c>
-      <c r="F10">
-        <f>D10*E10</f>
-        <v/>
+      <c r="F10" s="1" t="n">
+        <v>1.92</v>
       </c>
     </row>
     <row r="11">
@@ -729,9 +724,8 @@
       <c r="E11" t="n">
         <v>2</v>
       </c>
-      <c r="F11">
-        <f>D11*E11</f>
-        <v/>
+      <c r="F11" s="1" t="n">
+        <v>0.24</v>
       </c>
     </row>
     <row r="12">
@@ -756,9 +750,8 @@
       <c r="E12" t="n">
         <v>4</v>
       </c>
-      <c r="F12">
-        <f>D12*E12</f>
-        <v/>
+      <c r="F12" s="1" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="13">
@@ -783,6 +776,9 @@
       <c r="E13" t="n">
         <v>1</v>
       </c>
+      <c r="F13" s="1" t="n">
+        <v>280</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -806,9 +802,8 @@
       <c r="E14" t="n">
         <v>1</v>
       </c>
-      <c r="F14">
-        <f>D14*E14</f>
-        <v/>
+      <c r="F14" s="1" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="15">
@@ -833,9 +828,8 @@
       <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="F15">
-        <f>D15*E15</f>
-        <v/>
+      <c r="F15" s="1" t="n">
+        <v>3.8</v>
       </c>
     </row>
     <row r="16">
@@ -860,9 +854,8 @@
       <c r="E16" t="n">
         <v>3</v>
       </c>
-      <c r="F16">
-        <f>D16*E16</f>
-        <v/>
+      <c r="F16" s="1" t="n">
+        <v>11.4</v>
       </c>
     </row>
     <row r="17">
@@ -887,9 +880,8 @@
       <c r="E17" t="n">
         <v>1</v>
       </c>
-      <c r="F17">
-        <f>D17*E17</f>
-        <v/>
+      <c r="F17" s="1" t="n">
+        <v>3.8</v>
       </c>
     </row>
     <row r="18">
@@ -914,9 +906,8 @@
       <c r="E18" t="n">
         <v>1</v>
       </c>
-      <c r="F18">
-        <f>D18*E18</f>
-        <v/>
+      <c r="F18" s="1" t="n">
+        <v>3.8</v>
       </c>
     </row>
     <row r="19">
@@ -941,9 +932,8 @@
       <c r="E19" t="n">
         <v>2</v>
       </c>
-      <c r="F19">
-        <f>D19*E19</f>
-        <v/>
+      <c r="F19" s="1" t="n">
+        <v>7.6</v>
       </c>
     </row>
     <row r="20">
@@ -968,9 +958,8 @@
       <c r="E20" t="n">
         <v>2</v>
       </c>
-      <c r="F20">
-        <f>D20*E20</f>
-        <v/>
+      <c r="F20" s="1" t="n">
+        <v>7.6</v>
       </c>
     </row>
     <row r="21">
@@ -995,9 +984,8 @@
       <c r="E21" t="n">
         <v>1</v>
       </c>
-      <c r="F21">
-        <f>D21*E21</f>
-        <v/>
+      <c r="F21" s="1" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="22">
@@ -1118,9 +1106,8 @@
       <c r="E26" t="n">
         <v>1</v>
       </c>
-      <c r="F26">
-        <f>D26*E26</f>
-        <v/>
+      <c r="F26" s="1" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="27">
@@ -1241,9 +1228,8 @@
       <c r="E31" t="n">
         <v>2</v>
       </c>
-      <c r="F31">
-        <f>D31*E31</f>
-        <v/>
+      <c r="F31" s="1" t="n">
+        <v>8.4</v>
       </c>
     </row>
     <row r="32">
@@ -1316,9 +1302,8 @@
       <c r="E34" t="n">
         <v>1</v>
       </c>
-      <c r="F34">
-        <f>D34*E34</f>
-        <v/>
+      <c r="F34" s="1" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="35">
@@ -1439,9 +1424,8 @@
       <c r="E39" t="n">
         <v>1</v>
       </c>
-      <c r="F39">
-        <f>D39*E39</f>
-        <v/>
+      <c r="F39" s="1" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="40">
@@ -1538,9 +1522,8 @@
       <c r="E43" t="n">
         <v>1</v>
       </c>
-      <c r="F43">
-        <f>D43*E43</f>
-        <v/>
+      <c r="F43" s="1" t="n">
+        <v>4.2</v>
       </c>
     </row>
     <row r="44">
@@ -1685,9 +1668,8 @@
       <c r="E49" t="n">
         <v>1</v>
       </c>
-      <c r="F49">
-        <f>D49*E49</f>
-        <v/>
+      <c r="F49" s="1" t="n">
+        <v>6.5</v>
       </c>
     </row>
     <row r="50">
@@ -1784,9 +1766,8 @@
       <c r="E53" t="n">
         <v>1</v>
       </c>
-      <c r="F53">
-        <f>D53*E53</f>
-        <v/>
+      <c r="F53" s="1" t="n">
+        <v>1.6</v>
       </c>
     </row>
     <row r="54">
@@ -1811,9 +1792,8 @@
       <c r="E54" t="n">
         <v>1</v>
       </c>
-      <c r="F54">
-        <f>D54*E54</f>
-        <v/>
+      <c r="F54" s="1" t="n">
+        <v>1.6</v>
       </c>
     </row>
     <row r="55">
@@ -1838,9 +1818,8 @@
       <c r="E55" t="n">
         <v>1</v>
       </c>
-      <c r="F55">
-        <f>D55*E55</f>
-        <v/>
+      <c r="F55" s="1" t="n">
+        <v>0.08</v>
       </c>
     </row>
     <row r="56">
@@ -1849,9 +1828,8 @@
           <t>总计1平方辅料</t>
         </is>
       </c>
-      <c r="F56">
-        <f>SUM(F9:F55)</f>
-        <v/>
+      <c r="F56" s="1" t="n">
+        <v>376.2</v>
       </c>
     </row>
     <row r="57"/>
@@ -1874,9 +1852,11 @@
       <c r="D58" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="F58">
-        <f>D58*E58</f>
-        <v/>
+      <c r="E58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="1" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="59">
@@ -1898,9 +1878,11 @@
       <c r="D59" s="1" t="n">
         <v>185</v>
       </c>
-      <c r="F59">
-        <f>D59*E59</f>
-        <v/>
+      <c r="E59" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="1" t="n">
+        <v>185</v>
       </c>
     </row>
     <row r="60">
@@ -1909,9 +1891,8 @@
           <t>包材总计</t>
         </is>
       </c>
-      <c r="F60">
-        <f>SUM(F58:F59)+6</f>
-        <v/>
+      <c r="F60" s="1" t="n">
+        <v>207</v>
       </c>
     </row>
     <row r="61"/>
@@ -2223,9 +2204,8 @@
           <t>10平方整体用量总计共用辅料</t>
         </is>
       </c>
-      <c r="E79">
-        <f>SUM(E63:E78)</f>
-        <v/>
+      <c r="E79" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -2234,9 +2214,8 @@
           <t>10平方整体用量总计共用辅料，单价1平方</t>
         </is>
       </c>
-      <c r="E80">
-        <f>E79/10</f>
-        <v/>
+      <c r="E80" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="81"/>
@@ -2563,6 +2542,9 @@
       <c r="D2" s="1" t="n">
         <v>880</v>
       </c>
+      <c r="E2" s="1" t="n">
+        <v>880</v>
+      </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
@@ -2589,6 +2571,9 @@
       <c r="D3" s="1" t="n">
         <v>880</v>
       </c>
+      <c r="E3" s="1" t="n">
+        <v>880</v>
+      </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
@@ -2615,6 +2600,9 @@
       <c r="D4" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E4" s="1" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
@@ -2631,9 +2619,8 @@
       <c r="D5" s="1" t="n">
         <v>1.5</v>
       </c>
-      <c r="E5">
-        <f>E4/10</f>
-        <v/>
+      <c r="E5" s="1" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="6"/>
@@ -2656,6 +2643,9 @@
       <c r="D7" s="1" t="n">
         <v>0.08</v>
       </c>
+      <c r="E7" s="1" t="n">
+        <v>9.6</v>
+      </c>
       <c r="F7" t="n">
         <v>120</v>
       </c>
@@ -2682,6 +2672,9 @@
       <c r="D8" s="1" t="n">
         <v>0.12</v>
       </c>
+      <c r="E8" s="1" t="n">
+        <v>4.8</v>
+      </c>
       <c r="F8" t="n">
         <v>40</v>
       </c>
@@ -2708,6 +2701,9 @@
       <c r="D9" s="1" t="n">
         <v>0.08</v>
       </c>
+      <c r="E9" s="1" t="n">
+        <v>10.56</v>
+      </c>
       <c r="F9" t="n">
         <v>132</v>
       </c>
@@ -2734,6 +2730,9 @@
       <c r="D10" s="1" t="n">
         <v>0.12</v>
       </c>
+      <c r="E10" s="1" t="n">
+        <v>172.8</v>
+      </c>
       <c r="F10" t="n">
         <v>1440</v>
       </c>
@@ -2760,6 +2759,9 @@
       <c r="D11" s="1" t="n">
         <v>0.12</v>
       </c>
+      <c r="E11" s="1" t="n">
+        <v>3.36</v>
+      </c>
       <c r="F11" t="n">
         <v>28</v>
       </c>
@@ -2806,9 +2808,6 @@
           <t>插装发光二极管/红色/347椭圆/HZ-347PR3H0F1XE-X2/发光强度1000-1200mcd/波长620-625/电压1.7-2.1V/5mA/视角65℃/带卡口/VEN00061</t>
         </is>
       </c>
-      <c r="D13" s="1" t="n">
-        <v>1.5</v>
-      </c>
       <c r="F13" t="n">
         <v>92160</v>
       </c>
@@ -2832,9 +2831,6 @@
           <t>插装发光二极管/绿色/347椭圆/HZ-347PG3H0F1TE-X1/发光强度2300-2500mcd  2500-2800mcd两段50%比例混用/波长528-531 531-534两段50%比例混用/电压2.4-2.8V/5mA/视角65℃/带卡口/VEN00061</t>
         </is>
       </c>
-      <c r="D14" s="1" t="n">
-        <v>1.5</v>
-      </c>
       <c r="F14" t="n">
         <v>92160</v>
       </c>
@@ -2858,9 +2854,6 @@
           <t>插装发光二极管/蓝色/347椭圆/HZ-347PB3H0F1TE-X2/发光强度460-500mcd 500-550mcd/波长466-469nm 469-472nm两段50%比例混用/电压2.4-2.8V/5mA/视角65℃/带卡口/VEN00061</t>
         </is>
       </c>
-      <c r="D15" s="1" t="n">
-        <v>1.5</v>
-      </c>
       <c r="F15" t="n">
         <v>92160</v>
       </c>
@@ -2884,9 +2877,6 @@
           <t>P10.416底壳/CDKXB-YZMZ-B1/500*250*18 /VEN00452 PC+15%GF 本色</t>
         </is>
       </c>
-      <c r="D16" s="1" t="n">
-        <v>1.5</v>
-      </c>
       <c r="F16" t="n">
         <v>80</v>
       </c>
@@ -2910,9 +2900,6 @@
           <t>P10.416面罩/CDKXB-YZMZ-B2/250*250 /VEN00452 PC+15%GF 本色</t>
         </is>
       </c>
-      <c r="D17" s="1" t="n">
-        <v>1.5</v>
-      </c>
       <c r="F17" t="n">
         <v>160</v>
       </c>
@@ -2962,6 +2949,9 @@
       <c r="D19" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E19" s="1" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
@@ -2988,6 +2978,9 @@
       <c r="D20" s="1" t="n">
         <v>280</v>
       </c>
+      <c r="E20" s="1" t="n">
+        <v>1400</v>
+      </c>
       <c r="F20" t="n">
         <v>5</v>
       </c>
@@ -3014,6 +3007,9 @@
       <c r="D21" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E21" s="1" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
@@ -3040,6 +3036,9 @@
       <c r="D22" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E22" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="F22" t="n">
         <v>20</v>
       </c>
@@ -3066,6 +3065,9 @@
       <c r="D23" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E23" s="1" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
@@ -3092,6 +3094,9 @@
       <c r="D24" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E24" s="1" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
@@ -3118,6 +3123,9 @@
       <c r="D25" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E25" s="1" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
@@ -3144,6 +3152,9 @@
       <c r="D26" s="1" t="n">
         <v>3.8</v>
       </c>
+      <c r="E26" s="1" t="n">
+        <v>3.8</v>
+      </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
@@ -3170,6 +3181,9 @@
       <c r="D27" s="1" t="n">
         <v>0.28</v>
       </c>
+      <c r="E27" s="1" t="n">
+        <v>1.12</v>
+      </c>
       <c r="F27" t="n">
         <v>4</v>
       </c>
@@ -3196,6 +3210,9 @@
       <c r="D28" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E28" s="1" t="n">
+        <v>0.45</v>
+      </c>
       <c r="F28" t="n">
         <v>0.3</v>
       </c>
@@ -3222,6 +3239,9 @@
       <c r="D29" s="1" t="n">
         <v>2.5</v>
       </c>
+      <c r="E29" s="1" t="n">
+        <v>12.5</v>
+      </c>
       <c r="F29" t="n">
         <v>5</v>
       </c>
@@ -3248,6 +3268,9 @@
       <c r="D30" s="1" t="n">
         <v>3.8</v>
       </c>
+      <c r="E30" s="1" t="n">
+        <v>228</v>
+      </c>
       <c r="F30" t="n">
         <v>60</v>
       </c>
@@ -3274,6 +3297,9 @@
       <c r="D31" s="1" t="n">
         <v>3.8</v>
       </c>
+      <c r="E31" s="1" t="n">
+        <v>38</v>
+      </c>
       <c r="F31" t="n">
         <v>10</v>
       </c>
@@ -3300,6 +3326,9 @@
       <c r="D32" s="1" t="n">
         <v>3.8</v>
       </c>
+      <c r="E32" s="1" t="n">
+        <v>19</v>
+      </c>
       <c r="F32" t="n">
         <v>5</v>
       </c>
@@ -3326,6 +3355,9 @@
       <c r="D33" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E33" s="1" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
@@ -3352,6 +3384,9 @@
       <c r="D34" s="1" t="n">
         <v>4.5</v>
       </c>
+      <c r="E34" s="1" t="n">
+        <v>9</v>
+      </c>
       <c r="F34" t="n">
         <v>2</v>
       </c>
@@ -3378,6 +3413,9 @@
       <c r="D35" s="1" t="n">
         <v>4.5</v>
       </c>
+      <c r="E35" s="1" t="n">
+        <v>18</v>
+      </c>
       <c r="F35" t="n">
         <v>4</v>
       </c>
@@ -3404,6 +3442,9 @@
       <c r="D36" s="1" t="n">
         <v>3.8</v>
       </c>
+      <c r="E36" s="1" t="n">
+        <v>79.8</v>
+      </c>
       <c r="F36" t="n">
         <v>21</v>
       </c>
@@ -3430,6 +3471,9 @@
       <c r="D37" s="1" t="n">
         <v>3.8</v>
       </c>
+      <c r="E37" s="1" t="n">
+        <v>114</v>
+      </c>
       <c r="F37" t="n">
         <v>30</v>
       </c>
@@ -3456,6 +3500,9 @@
       <c r="D38" s="1" t="n">
         <v>0.08</v>
       </c>
+      <c r="E38" s="1" t="n">
+        <v>8</v>
+      </c>
       <c r="F38" t="n">
         <v>100</v>
       </c>
@@ -3482,6 +3529,9 @@
       <c r="D39" s="1" t="n">
         <v>2.5</v>
       </c>
+      <c r="E39" s="1" t="n">
+        <v>7.5</v>
+      </c>
       <c r="F39" t="n">
         <v>3</v>
       </c>
@@ -3508,6 +3558,9 @@
       <c r="D40" s="1" t="n">
         <v>2.5</v>
       </c>
+      <c r="E40" s="1" t="n">
+        <v>7.5</v>
+      </c>
       <c r="F40" t="n">
         <v>3</v>
       </c>
@@ -3534,6 +3587,9 @@
       <c r="D41" s="1" t="n">
         <v>6.5</v>
       </c>
+      <c r="E41" s="1" t="n">
+        <v>149.5</v>
+      </c>
       <c r="F41" t="n">
         <v>23</v>
       </c>
@@ -3560,6 +3616,9 @@
       <c r="D42" s="1" t="n">
         <v>6.5</v>
       </c>
+      <c r="E42" s="1" t="n">
+        <v>149.5</v>
+      </c>
       <c r="F42" t="n">
         <v>23</v>
       </c>
@@ -3586,6 +3645,9 @@
       <c r="D43" s="1" t="n">
         <v>6.5</v>
       </c>
+      <c r="E43" s="1" t="n">
+        <v>227.5</v>
+      </c>
       <c r="F43" t="n">
         <v>35</v>
       </c>
@@ -3612,6 +3674,9 @@
       <c r="D44" s="1" t="n">
         <v>2.5</v>
       </c>
+      <c r="E44" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="F44" t="n">
         <v>12</v>
       </c>
@@ -3638,6 +3703,9 @@
       <c r="D45" s="1" t="n">
         <v>1.5</v>
       </c>
+      <c r="E45" s="1" t="n">
+        <v>1.5</v>
+      </c>
       <c r="F45" t="n">
         <v>1</v>
       </c>
@@ -3664,6 +3732,9 @@
       <c r="D46" s="1" t="n">
         <v>0.28</v>
       </c>
+      <c r="E46" s="1" t="n">
+        <v>14</v>
+      </c>
       <c r="F46" t="n">
         <v>50</v>
       </c>
@@ -3690,6 +3761,9 @@
       <c r="D47" s="1" t="n">
         <v>0.28</v>
       </c>
+      <c r="E47" s="1" t="n">
+        <v>35.56</v>
+      </c>
       <c r="F47" t="n">
         <v>127</v>
       </c>
@@ -3716,6 +3790,9 @@
       <c r="D48" s="1" t="n">
         <v>0.28</v>
       </c>
+      <c r="E48" s="1" t="n">
+        <v>2.8</v>
+      </c>
       <c r="F48" t="n">
         <v>10</v>
       </c>
@@ -3742,6 +3819,9 @@
       <c r="D49" s="1" t="n">
         <v>0.28</v>
       </c>
+      <c r="E49" s="1" t="n">
+        <v>12.6</v>
+      </c>
       <c r="F49" t="n">
         <v>45</v>
       </c>
@@ -3768,6 +3848,9 @@
       <c r="D50" s="1" t="n">
         <v>0.28</v>
       </c>
+      <c r="E50" s="1" t="n">
+        <v>4.76</v>
+      </c>
       <c r="F50" t="n">
         <v>17</v>
       </c>
@@ -3794,6 +3877,9 @@
       <c r="D51" s="1" t="n">
         <v>0.35</v>
       </c>
+      <c r="E51" s="1" t="n">
+        <v>0.875</v>
+      </c>
       <c r="F51" t="n">
         <v>2.5</v>
       </c>
@@ -3820,6 +3906,9 @@
       <c r="D52" s="1" t="n">
         <v>1.2</v>
       </c>
+      <c r="E52" s="1" t="n">
+        <v>1.2</v>
+      </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
@@ -3846,6 +3935,9 @@
       <c r="D53" s="1" t="n">
         <v>1.2</v>
       </c>
+      <c r="E53" s="1" t="n">
+        <v>48</v>
+      </c>
       <c r="F53" t="n">
         <v>40</v>
       </c>
@@ -3872,6 +3964,9 @@
       <c r="D54" s="1" t="n">
         <v>1.2</v>
       </c>
+      <c r="E54" s="1" t="n">
+        <v>1.2</v>
+      </c>
       <c r="F54" t="n">
         <v>1</v>
       </c>
@@ -3898,6 +3993,9 @@
       <c r="D55" s="1" t="n">
         <v>1.2</v>
       </c>
+      <c r="E55" s="1" t="n">
+        <v>1.2</v>
+      </c>
       <c r="F55" t="n">
         <v>1</v>
       </c>
@@ -3924,6 +4022,9 @@
       <c r="D56" t="n">
         <v>0</v>
       </c>
+      <c r="E56" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="F56" t="n">
         <v>1</v>
       </c>
@@ -3932,9 +4033,8 @@
       </c>
     </row>
     <row r="57">
-      <c r="E57">
-        <f>SUM(E7:E56)</f>
-        <v/>
+      <c r="E57" s="1" t="n">
+        <v>2866.985</v>
       </c>
     </row>
     <row r="58">
@@ -3943,9 +4043,8 @@
           <t>1平方辅料单价</t>
         </is>
       </c>
-      <c r="E58">
-        <f>E57/10</f>
-        <v/>
+      <c r="E58" s="1" t="n">
+        <v>286.6985</v>
       </c>
     </row>
     <row r="59"/>
@@ -3968,6 +4067,9 @@
       <c r="D60" s="1" t="n">
         <v>28</v>
       </c>
+      <c r="E60" s="1" t="n">
+        <v>84</v>
+      </c>
       <c r="F60" t="n">
         <v>3</v>
       </c>
@@ -3994,6 +4096,9 @@
       <c r="D61" s="1" t="n">
         <v>28</v>
       </c>
+      <c r="E61" s="1" t="n">
+        <v>56</v>
+      </c>
       <c r="F61" t="n">
         <v>2</v>
       </c>
@@ -4002,9 +4107,8 @@
       </c>
     </row>
     <row r="62">
-      <c r="E62">
-        <f>SUM(E60:E61)</f>
-        <v/>
+      <c r="E62" s="1" t="n">
+        <v>140</v>
       </c>
     </row>
     <row r="63">
@@ -4013,9 +4117,8 @@
           <t>包材总计</t>
         </is>
       </c>
-      <c r="E63">
-        <f>E62/10+2</f>
-        <v/>
+      <c r="E63" s="1" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="64"/>
@@ -4038,6 +4141,9 @@
       <c r="D65" s="1" t="n">
         <v>22</v>
       </c>
+      <c r="E65" s="1" t="n">
+        <v>396</v>
+      </c>
       <c r="F65" t="n">
         <v>18</v>
       </c>
@@ -4064,6 +4170,9 @@
       <c r="D66" s="1" t="n">
         <v>22</v>
       </c>
+      <c r="E66" s="1" t="n">
+        <v>88</v>
+      </c>
       <c r="F66" t="n">
         <v>4</v>
       </c>
@@ -4090,6 +4199,9 @@
       <c r="D67" s="1" t="n">
         <v>0.18</v>
       </c>
+      <c r="E67" s="1" t="n">
+        <v>6.48</v>
+      </c>
       <c r="F67" t="n">
         <v>36</v>
       </c>
@@ -4116,6 +4228,9 @@
       <c r="D68" s="1" t="n">
         <v>0.12</v>
       </c>
+      <c r="E68" s="1" t="n">
+        <v>9.6</v>
+      </c>
       <c r="F68" t="n">
         <v>80</v>
       </c>
@@ -4142,6 +4257,9 @@
       <c r="D69" s="1" t="n">
         <v>0.12</v>
       </c>
+      <c r="E69" s="1" t="n">
+        <v>7.2</v>
+      </c>
       <c r="F69" t="n">
         <v>60</v>
       </c>
@@ -4168,6 +4286,9 @@
       <c r="D70" s="1" t="n">
         <v>0.55</v>
       </c>
+      <c r="E70" s="1" t="n">
+        <v>11</v>
+      </c>
       <c r="F70" t="n">
         <v>20</v>
       </c>
@@ -4194,6 +4315,9 @@
       <c r="D71" s="1" t="n">
         <v>0.55</v>
       </c>
+      <c r="E71" s="1" t="n">
+        <v>30.8</v>
+      </c>
       <c r="F71" t="n">
         <v>56</v>
       </c>
@@ -4220,6 +4344,9 @@
       <c r="D72" s="1" t="n">
         <v>0.12</v>
       </c>
+      <c r="E72" s="1" t="n">
+        <v>3.84</v>
+      </c>
       <c r="F72" t="n">
         <v>32</v>
       </c>
@@ -4228,9 +4355,8 @@
       </c>
     </row>
     <row r="73">
-      <c r="E73">
-        <f>SUM(E65:E72)</f>
-        <v/>
+      <c r="E73" s="1" t="n">
+        <v>552.92</v>
       </c>
     </row>
     <row r="74">
@@ -4242,9 +4368,8 @@
       <c r="D74" s="1" t="n">
         <v>0.15</v>
       </c>
-      <c r="E74">
-        <f>E73/10+5</f>
-        <v/>
+      <c r="E74" s="1" t="n">
+        <v>60.292</v>
       </c>
     </row>
   </sheetData>
@@ -4400,13 +4525,11 @@
         <f>J3*I3</f>
         <v/>
       </c>
-      <c r="N3">
-        <f>压铸铝辅材!F60</f>
-        <v/>
-      </c>
-      <c r="O3">
-        <f>压铸铝辅材!F56+压铸铝辅材!E80+20</f>
-        <v/>
+      <c r="N3" s="1" t="n">
+        <v>207</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>396.2</v>
       </c>
       <c r="P3">
         <f>G3+H3+K3+L3+M3+N3+O3</f>
@@ -4530,13 +4653,11 @@
         <f>J5*I5</f>
         <v/>
       </c>
-      <c r="N5">
-        <f>铁箱辅材!E63</f>
-        <v/>
-      </c>
-      <c r="O5">
-        <f>铁箱辅材!E58+20</f>
-        <v/>
+      <c r="N5" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="1" t="n">
+        <v>306.6985</v>
       </c>
       <c r="P5">
         <f>G5+H5+K5+L5+M5+N5+O5</f>

</xml_diff>

<commit_message>
Make Chuangdi quote skills self-contained without the original workbook.
Embed morph formulas and hardcoded constants in skills, require the three-file input set only, migrate bracket/PSU pricing into the accounting book, and add product-scope plus demo-rule docs for the POC run.
</commit_message>
<xml_diff>
--- a/chuangdi/数据/核算口径表-演示.xlsx
+++ b/chuangdi/数据/核算口径表-演示.xlsx
@@ -10,7 +10,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="压铸铝辅材" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="铁箱辅材" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每平米收口" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="箱体" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="电源" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="支架" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安装抱箍和螺钉" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每平米收口" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,14 +451,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>本文件整理自大模组核算原表，定位是造价演算底稿中的「数量口径 + 辅材 BOM」，不是又一份模组/箱体价目。</t>
+          <t>本文件整理自大模组核算原表：辅材 BOM、每平米收口结构、箱体/电源/支架/抱箍价目。「每平米收口」样例行是历史底稿，项目报价由 Agent 按招标+规格+本表规则重算本项目收口，不是样例×面积。</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Agent 报价三件套：规格单价表（大件单价）+ 本表 BOM/收口（小件摊到每平米）+ 计价 skill（公式骨架）。</t>
+          <t>三件套：规格单价表（模组/灯珠/套件及物理箱 SKU）+ 本表（BOM、收口结构、元/㎡箱体与电源/支架/抱箍价目）+ 计价 skill。详见方案/场景演示建议口径.md、原表公式与经验配量确认.md。</t>
         </is>
       </c>
     </row>
@@ -468,28 +472,35 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>每平米收口：保留点间距×箱体材料行、1㎡模组数量、电源数量；包材/辅材公式引用辅材表。模组单价、箱体单价、电源单价列留空——取自规格单价表，勿在此另维护一份。</t>
+          <t>每平米收口：保留结构与对辅材/箱体/电源的公式引用；模组单价列正式稿留空（取规格单价表）。表内「1㎡模组数量」「常规电源数量」为样例/待成本确认的经验位，不作未确认的项目默认取数。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>公式骨架相对固定；BOM 明细与常数加价（如辅材公式中的 +20）由成本岗维护，改后同步 skill。</t>
+          <t>价目页「箱体」「电源」「支架」「安装抱箍和螺钉」自原表迁入；正式稿单价空/0 由成本维护。规格单价表「箱体单价」仅作物料核对，平方单价中的箱体元/㎡以本册「箱体」为准。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>招标报价用抄录面积，不依赖原屏体清单样例长宽。供应商名不转入。</t>
+          <t>不转入屏体清单样例页、压铸铝控制箱。招标用抄录面积。供应商名不转入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BOM 明细与常数加价（如辅材 +20）由成本岗维护，改后同步 skill。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>【演示副本】已为辅材 BOM 空单价填模拟数，并按公式骨架滚出行合计与 1㎡ 辅料/包材汇总（黄底）。正式稿大件单价仍应留空、取自规格单价表；正式稿汇总格保留公式，须在 Excel 中打开计算或由人维护滚出值。本文件不是创迪成本。</t>
+          <t>【演示副本】辅材 BOM、箱体/电源/支架/抱箍价目已填模拟单价（黄底）并滚出可读汇总。「常规电源数量」等为演示维护示意，供 POC 重算本项目收口；不是未确认的正式成本定额。本文件不是创迪采购价。正式稿单价由成本维护；项目报价按招标+规格重算，非样例×面积。</t>
         </is>
       </c>
     </row>
@@ -4383,6 +4394,3084 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>箱体单价</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>单位</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>箱体单价</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>配件单价</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>综合单价</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>压铸铝箱体</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>990</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>1030</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>不含包边</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>镀锌钢板箱体</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>830</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>870</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>不含包边</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>镀锌钢板箱体</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>㎡</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>830</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>870</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>含包边</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>电源单价</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>规格</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>功率因素</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>温度</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>单位</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>单价</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>100W/5V</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>100W/5V</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>100W/5V</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>低温</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>110W/3.2V+3.8V</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>110W/3.2V+3.8V</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>低温</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>175W/3.2V+3.8V</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>175W/3.2V+3.8V</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>低温</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>200W/5V</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>44厚款</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>200W/5V</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>200W/5V</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>低温</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>175W/3.2V+3.8V</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>175W/3.2V+3.8V</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>低温</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>300W/5V</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>300W/5V</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>常规</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>300W/5V</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>高功率因素</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>低温</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="n">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>支架单价</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>单位</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>支架单价</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>螺钉配件单价</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>综合单价</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>收费大棚吊装吊架</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>平方</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>400</v>
+      </c>
+      <c r="F3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>收费大棚背部支架</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>平方</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>路段1米高支撑架</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>平方</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>110</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>路段2米高支撑架</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>平方</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>160</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>路段1㎡支撑架</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>400</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>路段2㎡支撑架</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>400</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>路段4㎡支撑架</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>400</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>悬臂含走道支架</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>230</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>3.2*1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>悬臂含走道支架</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>230</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>4*2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>洞内屏2支架2节支架</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E12">
+        <f>E24</f>
+        <v/>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G12">
+        <f>E12+F12</f>
+        <v/>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>含膨胀螺栓</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>洞内屏2支架3节支架</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E13">
+        <f>E43</f>
+        <v/>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13">
+        <f>E13+F13</f>
+        <v/>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>含膨胀螺栓</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>洞内屏3支架3节支架</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E14">
+        <f>E63</f>
+        <v/>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G14">
+        <f>E14+F14</f>
+        <v/>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>含膨胀螺栓</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>洞内侧壁1.6*3.2支架</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E15">
+        <f>400*1.6*3.2</f>
+        <v/>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G15">
+        <f>E15+F15</f>
+        <v/>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>含膨胀螺栓</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>洞内侧壁1*2支架</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="E16">
+        <f>400*2</f>
+        <v/>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G16">
+        <f>E16+F16</f>
+        <v/>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>含膨胀螺栓</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>服务区</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>平方</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>600</v>
+      </c>
+      <c r="F17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" s="1" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>洞内两支架两节</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BOM层级</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>子项物料编码</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>物料名称</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>含税单价</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>价税合计</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>标准用量</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>实际数量</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>替代方式</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>3000001603</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>洞内拱顶可变信息标志（双色)/P25 2R1G 200*200/CDCKB25+DN01/2500*1300*200/SGCC=1.5  蓝灰色(钣金箱体）2025-BS013</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>10413.57</v>
+      </c>
+      <c r="E21" t="n">
+        <v>10413.57</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>10414.57</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1700000482</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>洞内吊架顶安装板/CDTPJ-AZL-C2B/280*200*295/Q235=20MM 热镀锌本色</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>167.96</v>
+      </c>
+      <c r="E22" t="n">
+        <v>335.92</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>337.92</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1700000107</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>洞内吊架下安装支架/CDTPJ-AZL-C4/300*200*300/槽钢+Q235 热镀锌本色</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>131.12</v>
+      </c>
+      <c r="E23" t="n">
+        <v>262.24</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="1" t="n">
+        <v>264.24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2支架成本总计</t>
+        </is>
+      </c>
+      <c r="E24">
+        <f>SUM(E22:E23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>洞内两支架两节</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1600000048</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>不锈钢弹垫/M24/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4</v>
+      </c>
+      <c r="G27" s="1" t="n">
+        <v>6.28</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1600000054</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>不锈钢平垫/M24/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8</v>
+      </c>
+      <c r="G28" s="1" t="n">
+        <v>13.68</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1600000007</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>螺母/M24/不锈钢；A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="E29" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="F29" t="n">
+        <v>8</v>
+      </c>
+      <c r="G29" s="1" t="n">
+        <v>26.8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1600000042</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>外六角螺栓/M24*80/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="1" t="n">
+        <v>36.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1600000041</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>外六角螺栓/M18*60/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E31" t="n">
+        <v>26.88</v>
+      </c>
+      <c r="F31" t="n">
+        <v>8</v>
+      </c>
+      <c r="G31" s="1" t="n">
+        <v>34.88</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1600000047</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>不锈钢弹垫/M18/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="F32" t="n">
+        <v>8</v>
+      </c>
+      <c r="G32" s="1" t="n">
+        <v>9.76</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1600000053</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>不锈钢平垫/M18/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E33" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="F33" t="n">
+        <v>16</v>
+      </c>
+      <c r="G33" s="1" t="n">
+        <v>21.28</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1600000006</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>螺母/M18/不锈钢；A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E34" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="F34" t="n">
+        <v>8</v>
+      </c>
+      <c r="G34" s="1" t="n">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>总计螺钉</t>
+        </is>
+      </c>
+      <c r="E35">
+        <f>SUM(E27:E34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>洞内两支架三节</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BOM层级</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>子项物料编码</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>物料名称</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>含税单价</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>价税合计</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>标准用量</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>实际数量</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>3000001744</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>洞内拱顶可变信息标志（双色)/P25 2R1G 400*200/CDCKB25+DN01/2500*1300*200/SGCC=1.5 蓝灰色(钣金箱体）2025-S561</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>10132.8</v>
+      </c>
+      <c r="E39" t="n">
+        <v>10132.8</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="1" t="n">
+        <v>10133.8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1700000482</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>洞内吊架顶安装板/CDTPJ-AZL-C2B/280*200*295/Q235=20MM 热镀锌本色</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>167.96</v>
+      </c>
+      <c r="E40" t="n">
+        <v>335.92</v>
+      </c>
+      <c r="F40" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" s="1" t="n">
+        <v>337.92</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1700000107</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>洞内吊架下安装支架/CDTPJ-AZL-C4/300*200*300/槽钢+Q235 热镀锌本色</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>131.12</v>
+      </c>
+      <c r="E41" t="n">
+        <v>262.24</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" s="1" t="n">
+        <v>264.24</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1700000106</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>洞内吊架中间调节槽钢/CDTPJ-AZL-C3/120*53*450/槽钢 热镀锌本色</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>45.799999</v>
+      </c>
+      <c r="E42" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="1" t="n">
+        <v>93.59999999999999</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>3件套支架总计</t>
+        </is>
+      </c>
+      <c r="E43">
+        <f>SUM(E40:E42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>洞内两支架三节</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1600000041</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>外六角螺栓/M18*60/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E45" t="n">
+        <v>26.88</v>
+      </c>
+      <c r="F45" t="n">
+        <v>8</v>
+      </c>
+      <c r="G45" s="1" t="n">
+        <v>34.88</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1600000047</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>不锈钢弹垫/M18/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="F46" t="n">
+        <v>8</v>
+      </c>
+      <c r="G46" s="1" t="n">
+        <v>9.76</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1600000053</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>不锈钢平垫/M18/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E47" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="F47" t="n">
+        <v>16</v>
+      </c>
+      <c r="G47" s="1" t="n">
+        <v>21.28</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1600000006</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>螺母/M18/不锈钢；A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E48" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="F48" t="n">
+        <v>8</v>
+      </c>
+      <c r="G48" s="1" t="n">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1600000048</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>不锈钢弹垫/M24/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E49" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="F49" t="n">
+        <v>8</v>
+      </c>
+      <c r="G49" s="1" t="n">
+        <v>12.56</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1600000054</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>不锈钢平垫/M24/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="E50" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="F50" t="n">
+        <v>16</v>
+      </c>
+      <c r="G50" s="1" t="n">
+        <v>27.36</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1600000007</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>螺母/M24/不锈钢；A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="E51" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="F51" t="n">
+        <v>16</v>
+      </c>
+      <c r="G51" s="1" t="n">
+        <v>53.6</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1600000042</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>外六角螺栓/M24*80/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E52" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="F52" t="n">
+        <v>8</v>
+      </c>
+      <c r="G52" s="1" t="n">
+        <v>72.8</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>3件套螺钉总计</t>
+        </is>
+      </c>
+      <c r="E53">
+        <f>SUM(E45:E52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>洞内三支架三节</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BOM层级</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>子项物料编码</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>物料名称</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>含税单价</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>价税合计</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>标准用量</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>实际数量</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>3000001744</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>洞内拱顶可变信息标志（双色)/P25 2R1G 400*200/CDCKB25+DN01/2500*1300*200/SGCC=1.5 蓝灰色(钣金箱体）2025-S561</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>10132.8</v>
+      </c>
+      <c r="E59" t="n">
+        <v>10132.8</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="1" t="n">
+        <v>10133.8</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1700000482</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>洞内吊架顶安装板/CDTPJ-AZL-C2B/280*200*295/Q235=20MM 热镀锌本色</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>167.96</v>
+      </c>
+      <c r="E60">
+        <f>D60*F60</f>
+        <v/>
+      </c>
+      <c r="F60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G60" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1700000107</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>洞内吊架下安装支架/CDTPJ-AZL-C4/300*200*300/槽钢+Q235 热镀锌本色</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>131.12</v>
+      </c>
+      <c r="E61">
+        <f>F61*D61</f>
+        <v/>
+      </c>
+      <c r="F61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G61" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1700000106</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>洞内吊架中间调节槽钢/CDTPJ-AZL-C3/120*53*450/槽钢 热镀锌本色</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>86</v>
+      </c>
+      <c r="E62">
+        <f>D62*F62</f>
+        <v/>
+      </c>
+      <c r="F62" t="n">
+        <v>3</v>
+      </c>
+      <c r="G62" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>3件套支架总计</t>
+        </is>
+      </c>
+      <c r="E63">
+        <f>SUM(E60:E62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>洞内三支架三节</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1600000041</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>外六角螺栓/M18*60/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="E65">
+        <f>D65*F65</f>
+        <v/>
+      </c>
+      <c r="F65" t="n">
+        <v>12</v>
+      </c>
+      <c r="G65">
+        <f>F65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1600000047</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>不锈钢弹垫/M18/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E66">
+        <f>D66*F66</f>
+        <v/>
+      </c>
+      <c r="F66" t="n">
+        <v>12</v>
+      </c>
+      <c r="G66">
+        <f>F66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1600000053</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>不锈钢平垫/M18/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E67">
+        <f>D67*F67</f>
+        <v/>
+      </c>
+      <c r="F67" t="n">
+        <v>24</v>
+      </c>
+      <c r="G67">
+        <f>F67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1600000006</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>螺母/M18/不锈钢；A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E68">
+        <f>D68*F68</f>
+        <v/>
+      </c>
+      <c r="F68" t="n">
+        <v>12</v>
+      </c>
+      <c r="G68">
+        <f>F68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1600000048</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>不锈钢弹垫/M24/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E69">
+        <f>D69*F69</f>
+        <v/>
+      </c>
+      <c r="F69" t="n">
+        <v>12</v>
+      </c>
+      <c r="G69">
+        <f>F69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1600000054</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>不锈钢平垫/M24/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="E70">
+        <f>D70*F70</f>
+        <v/>
+      </c>
+      <c r="F70" t="n">
+        <v>24</v>
+      </c>
+      <c r="G70">
+        <f>F70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1600000007</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>螺母/M24/不锈钢；A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="E71">
+        <f>D71*F71</f>
+        <v/>
+      </c>
+      <c r="F71" t="n">
+        <v>24</v>
+      </c>
+      <c r="G71">
+        <f>F71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1600000042</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>外六角螺栓/M24*80/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E72">
+        <f>D72*F72</f>
+        <v/>
+      </c>
+      <c r="F72" t="n">
+        <v>12</v>
+      </c>
+      <c r="G72">
+        <f>F72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>3件套螺钉总计</t>
+        </is>
+      </c>
+      <c r="E73">
+        <f>SUM(E65:E72)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>安装抱箍和螺钉单价</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>抱箍数量</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>抱箍单价</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>抱箍合计</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>抱箍数量</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>几字安装件单价</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>几字安装件合计</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>螺钉配件数量</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>螺钉配件单价</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>螺钉配件合计</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>综合价格</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>收费大棚吊装吊架</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>收费大棚背部支架</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>路段1米高支撑架</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>路段2米高支撑架</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>路段1㎡支撑架</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K7" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>路段2㎡支撑架</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K8" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>悬臂含走道支架3.2*1.6</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>悬臂含走道支架4*2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>洞内屏2支架2节支架</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>洞内屏2支架3节支架</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H12" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K12" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>洞内屏3支架3节支架</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K13" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L13" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>洞内侧壁1.6*3.2支架</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H14" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K14" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L14" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>洞内侧壁1*2支架</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K15" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" s="1" t="n">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Q50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -4508,12 +7597,11 @@
       <c r="F3" s="1" t="n">
         <v>199.33</v>
       </c>
-      <c r="G3">
-        <f>E3*F3</f>
-        <v/>
+      <c r="G3" s="1" t="n">
+        <v>1594.64</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>990</v>
+        <v>1030</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
@@ -4521,9 +7609,8 @@
       <c r="J3" s="1" t="n">
         <v>72</v>
       </c>
-      <c r="K3">
-        <f>J3*I3</f>
-        <v/>
+      <c r="K3" s="1" t="n">
+        <v>144</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>207</v>
@@ -4531,13 +7618,12 @@
       <c r="O3" s="1" t="n">
         <v>396.2</v>
       </c>
-      <c r="P3">
-        <f>G3+H3+K3+L3+M3+N3+O3</f>
-        <v/>
+      <c r="P3" s="1" t="n">
+        <v>3371.84</v>
       </c>
       <c r="Q3" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -4564,17 +7650,15 @@
         <f>E4*F4</f>
         <v/>
       </c>
-      <c r="H4">
-        <f>H3</f>
-        <v/>
+      <c r="H4" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I4">
         <f>I3</f>
         <v/>
       </c>
-      <c r="J4">
-        <f>J3</f>
-        <v/>
+      <c r="J4" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K4">
         <f>J4*I4</f>
@@ -4596,13 +7680,12 @@
         <f>O3</f>
         <v/>
       </c>
-      <c r="P4">
-        <f>G4+H4+K4+L4+M4+N4+O4</f>
-        <v/>
+      <c r="P4" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q4" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -4631,27 +7714,23 @@
       <c r="E5" t="n">
         <v>8</v>
       </c>
-      <c r="F5">
-        <f>F3</f>
-        <v/>
-      </c>
-      <c r="G5">
-        <f>E5*F5</f>
-        <v/>
+      <c r="F5" s="1" t="n">
+        <v>199.33</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>1594.64</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>760</v>
+        <v>870</v>
       </c>
       <c r="I5" t="n">
         <v>2</v>
       </c>
-      <c r="J5">
-        <f>J3</f>
-        <v/>
-      </c>
-      <c r="K5">
-        <f>J5*I5</f>
-        <v/>
+      <c r="J5" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>144</v>
       </c>
       <c r="N5" s="1" t="n">
         <v>16</v>
@@ -4659,13 +7738,12 @@
       <c r="O5" s="1" t="n">
         <v>306.6985</v>
       </c>
-      <c r="P5">
-        <f>G5+H5+K5+L5+M5+N5+O5</f>
-        <v/>
+      <c r="P5" s="1" t="n">
+        <v>2931.34</v>
       </c>
       <c r="Q5" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -4685,25 +7763,22 @@
         <f>E5</f>
         <v/>
       </c>
-      <c r="F6">
-        <f>F4</f>
-        <v/>
+      <c r="F6" s="1" t="n">
+        <v>213.33</v>
       </c>
       <c r="G6">
         <f>E6*F6</f>
         <v/>
       </c>
-      <c r="H6">
-        <f>H5</f>
-        <v/>
+      <c r="H6" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I6">
         <f>I5</f>
         <v/>
       </c>
-      <c r="J6">
-        <f>J5</f>
-        <v/>
+      <c r="J6" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K6">
         <f>J6*I6</f>
@@ -4725,13 +7800,12 @@
         <f>O5</f>
         <v/>
       </c>
-      <c r="P6">
-        <f>G6+H6+K6+L6+M6+N6+O6</f>
-        <v/>
+      <c r="P6" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q6" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -4857,13 +7931,11 @@
       <c r="F9" s="1" t="n">
         <v>175</v>
       </c>
-      <c r="G9">
-        <f>E9*F9</f>
-        <v/>
-      </c>
-      <c r="H9">
-        <f>H3</f>
-        <v/>
+      <c r="G9" s="1" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I9" t="n">
         <v>2</v>
@@ -4871,9 +7943,8 @@
       <c r="J9" s="1" t="n">
         <v>72</v>
       </c>
-      <c r="K9">
-        <f>J9*I9</f>
-        <v/>
+      <c r="K9" s="1" t="n">
+        <v>144</v>
       </c>
       <c r="L9">
         <f>L3</f>
@@ -4891,13 +7962,12 @@
         <f>O3</f>
         <v/>
       </c>
-      <c r="P9">
-        <f>G9+H9+K9+L9+M9+N9+O9</f>
-        <v/>
+      <c r="P9" s="1" t="n">
+        <v>2574</v>
       </c>
       <c r="Q9" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -4919,21 +7989,18 @@
       <c r="F10" s="1" t="n">
         <v>189</v>
       </c>
-      <c r="G10">
-        <f>E10*F10</f>
-        <v/>
-      </c>
-      <c r="H10">
-        <f>H9</f>
-        <v/>
+      <c r="G10" s="1" t="n">
+        <v>1512</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I10">
         <f>I9</f>
         <v/>
       </c>
-      <c r="J10">
-        <f>J9</f>
-        <v/>
+      <c r="J10" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K10">
         <f>J10*I10</f>
@@ -4955,13 +8022,12 @@
         <f>O9</f>
         <v/>
       </c>
-      <c r="P10">
-        <f>G10+H10+K10+L10+M10+N10+O10</f>
-        <v/>
+      <c r="P10" s="1" t="n">
+        <v>2542</v>
       </c>
       <c r="Q10" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -4983,21 +8049,18 @@
       <c r="F11" s="1" t="n">
         <v>175</v>
       </c>
-      <c r="G11">
-        <f>E11*F11</f>
-        <v/>
-      </c>
-      <c r="H11">
-        <f>H10</f>
-        <v/>
+      <c r="G11" s="1" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I11">
         <f>I10</f>
         <v/>
       </c>
-      <c r="J11">
-        <f>J10</f>
-        <v/>
+      <c r="J11" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K11">
         <f>J11*I11</f>
@@ -5019,13 +8082,12 @@
         <f>O10</f>
         <v/>
       </c>
-      <c r="P11">
-        <f>G11+H11+K11+L11+M11+N11+O11</f>
-        <v/>
+      <c r="P11" s="1" t="n">
+        <v>2430</v>
       </c>
       <c r="Q11" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5052,17 +8114,15 @@
         <f>E12*F12</f>
         <v/>
       </c>
-      <c r="H12">
-        <f>H11</f>
-        <v/>
+      <c r="H12" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I12">
         <f>I11</f>
         <v/>
       </c>
-      <c r="J12">
-        <f>J11</f>
-        <v/>
+      <c r="J12" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K12">
         <f>J12*I12</f>
@@ -5084,13 +8144,12 @@
         <f>O11</f>
         <v/>
       </c>
-      <c r="P12">
-        <f>G12+H12+K12+L12+M12+N12+O12</f>
-        <v/>
+      <c r="P12" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q12" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5119,25 +8178,21 @@
       <c r="E13" t="n">
         <v>8</v>
       </c>
-      <c r="F13">
-        <f>F9</f>
-        <v/>
-      </c>
-      <c r="G13">
-        <f>E13*F13</f>
-        <v/>
-      </c>
-      <c r="H13">
-        <f>H5</f>
-        <v/>
+      <c r="F13" s="1" t="n">
+        <v>175</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I13">
         <f>I12</f>
         <v/>
       </c>
-      <c r="J13">
-        <f>J12</f>
-        <v/>
+      <c r="J13" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K13">
         <f>J13*I13</f>
@@ -5159,13 +8214,12 @@
         <f>O5</f>
         <v/>
       </c>
-      <c r="P13">
-        <f>G13+H13+K13+L13+M13+N13+O13</f>
-        <v/>
+      <c r="P13" s="1" t="n">
+        <v>2270</v>
       </c>
       <c r="Q13" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5184,25 +8238,21 @@
       <c r="E14" t="n">
         <v>8</v>
       </c>
-      <c r="F14">
-        <f>F10</f>
-        <v/>
-      </c>
-      <c r="G14">
-        <f>E14*F14</f>
-        <v/>
-      </c>
-      <c r="H14">
-        <f>H13</f>
-        <v/>
+      <c r="F14" s="1" t="n">
+        <v>189</v>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>1512</v>
+      </c>
+      <c r="H14" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I14">
         <f>I13</f>
         <v/>
       </c>
-      <c r="J14">
-        <f>J13</f>
-        <v/>
+      <c r="J14" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K14">
         <f>J14*I14</f>
@@ -5224,13 +8274,12 @@
         <f>O13</f>
         <v/>
       </c>
-      <c r="P14">
-        <f>G14+H14+K14+L14+M14+N14+O14</f>
-        <v/>
+      <c r="P14" s="1" t="n">
+        <v>2382</v>
       </c>
       <c r="Q14" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5249,25 +8298,21 @@
       <c r="E15" t="n">
         <v>8</v>
       </c>
-      <c r="F15">
-        <f>F11</f>
-        <v/>
-      </c>
-      <c r="G15">
-        <f>E15*F15</f>
-        <v/>
-      </c>
-      <c r="H15">
-        <f>H14</f>
-        <v/>
+      <c r="F15" s="1" t="n">
+        <v>175</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I15">
         <f>I14</f>
         <v/>
       </c>
-      <c r="J15">
-        <f>J14</f>
-        <v/>
+      <c r="J15" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K15">
         <f>J15*I15</f>
@@ -5289,13 +8334,12 @@
         <f>O14</f>
         <v/>
       </c>
-      <c r="P15">
-        <f>G15+H15+K15+L15+M15+N15+O15</f>
-        <v/>
+      <c r="P15" s="1" t="n">
+        <v>2270</v>
       </c>
       <c r="Q15" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5315,25 +8359,22 @@
         <f>E13</f>
         <v/>
       </c>
-      <c r="F16">
-        <f>F12</f>
-        <v/>
+      <c r="F16" s="1" t="n">
+        <v>189</v>
       </c>
       <c r="G16">
         <f>E16*F16</f>
         <v/>
       </c>
-      <c r="H16">
-        <f>H15</f>
-        <v/>
+      <c r="H16" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I16">
         <f>I15</f>
         <v/>
       </c>
-      <c r="J16">
-        <f>J15</f>
-        <v/>
+      <c r="J16" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K16">
         <f>J16*I16</f>
@@ -5355,13 +8396,12 @@
         <f>O15</f>
         <v/>
       </c>
-      <c r="P16">
-        <f>G16+H16+K16+L16+M16+N16+O16</f>
-        <v/>
+      <c r="P16" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q16" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5487,13 +8527,11 @@
       <c r="F19" s="1" t="n">
         <v>166.17</v>
       </c>
-      <c r="G19">
-        <f>E19*F19</f>
-        <v/>
-      </c>
-      <c r="H19">
-        <f>H3</f>
-        <v/>
+      <c r="G19" s="1" t="n">
+        <v>1329.36</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I19" t="n">
         <v>2</v>
@@ -5501,9 +8539,8 @@
       <c r="J19" s="1" t="n">
         <v>72</v>
       </c>
-      <c r="K19">
-        <f>J19*I19</f>
-        <v/>
+      <c r="K19" s="1" t="n">
+        <v>144</v>
       </c>
       <c r="L19">
         <f>L3</f>
@@ -5521,13 +8558,12 @@
         <f>O3</f>
         <v/>
       </c>
-      <c r="P19">
-        <f>G19+H19+K19+L19+M19+N19+O19</f>
-        <v/>
+      <c r="P19" s="1" t="n">
+        <v>2503.36</v>
       </c>
       <c r="Q19" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5554,17 +8590,15 @@
         <f>E20*F20</f>
         <v/>
       </c>
-      <c r="H20">
-        <f>H19</f>
-        <v/>
+      <c r="H20" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I20">
         <f>I19</f>
         <v/>
       </c>
-      <c r="J20">
-        <f>J19</f>
-        <v/>
+      <c r="J20" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K20">
         <f>J20*I20</f>
@@ -5586,13 +8620,12 @@
         <f>O19</f>
         <v/>
       </c>
-      <c r="P20">
-        <f>G20+H20+K20+L20+M20+N20+O20</f>
-        <v/>
+      <c r="P20" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q20" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5619,17 +8652,15 @@
         <f>E21*F21</f>
         <v/>
       </c>
-      <c r="H21">
-        <f>H20</f>
-        <v/>
+      <c r="H21" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I21">
         <f>I20</f>
         <v/>
       </c>
-      <c r="J21">
-        <f>J20</f>
-        <v/>
+      <c r="J21" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K21">
         <f>J21*I21</f>
@@ -5651,13 +8682,12 @@
         <f>O20</f>
         <v/>
       </c>
-      <c r="P21">
-        <f>G21+H21+K21+L21+M21+N21+O21</f>
-        <v/>
+      <c r="P21" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q21" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5687,25 +8717,22 @@
         <f>E21</f>
         <v/>
       </c>
-      <c r="F22">
-        <f>F19</f>
-        <v/>
+      <c r="F22" s="1" t="n">
+        <v>166.17</v>
       </c>
       <c r="G22">
         <f>E22*F22</f>
         <v/>
       </c>
-      <c r="H22">
-        <f>H5</f>
-        <v/>
+      <c r="H22" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I22">
         <f>I21</f>
         <v/>
       </c>
-      <c r="J22">
-        <f>J21</f>
-        <v/>
+      <c r="J22" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K22">
         <f>J22*I22</f>
@@ -5727,13 +8754,12 @@
         <f>O5</f>
         <v/>
       </c>
-      <c r="P22">
-        <f>G22+H22+K22+L22+M22+N22+O22</f>
-        <v/>
+      <c r="P22" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q22" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5753,25 +8779,22 @@
         <f>E22</f>
         <v/>
       </c>
-      <c r="F23">
-        <f>F20</f>
-        <v/>
+      <c r="F23" s="1" t="n">
+        <v>152.17</v>
       </c>
       <c r="G23">
         <f>E23*F23</f>
         <v/>
       </c>
-      <c r="H23">
-        <f>H22</f>
-        <v/>
+      <c r="H23" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I23">
         <f>I22</f>
         <v/>
       </c>
-      <c r="J23">
-        <f>J22</f>
-        <v/>
+      <c r="J23" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K23">
         <f>J23*I23</f>
@@ -5793,13 +8816,12 @@
         <f>O22</f>
         <v/>
       </c>
-      <c r="P23">
-        <f>G23+H23+K23+L23+M23+N23+O23</f>
-        <v/>
+      <c r="P23" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q23" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5819,25 +8841,22 @@
         <f>E23</f>
         <v/>
       </c>
-      <c r="F24">
-        <f>F21</f>
-        <v/>
+      <c r="F24" s="1" t="n">
+        <v>166.17</v>
       </c>
       <c r="G24">
         <f>E24*F24</f>
         <v/>
       </c>
-      <c r="H24">
-        <f>H23</f>
-        <v/>
+      <c r="H24" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I24">
         <f>I23</f>
         <v/>
       </c>
-      <c r="J24">
-        <f>J23</f>
-        <v/>
+      <c r="J24" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K24">
         <f>J24*I24</f>
@@ -5859,13 +8878,12 @@
         <f>O23</f>
         <v/>
       </c>
-      <c r="P24">
-        <f>G24+H24+K24+L24+M24+N24+O24</f>
-        <v/>
+      <c r="P24" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q24" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -5991,13 +9009,11 @@
       <c r="F27" s="1" t="n">
         <v>133.2</v>
       </c>
-      <c r="G27">
-        <f>E27*F27</f>
-        <v/>
-      </c>
-      <c r="H27">
-        <f>H3</f>
-        <v/>
+      <c r="G27" s="1" t="n">
+        <v>1065.6</v>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I27">
         <f>I3</f>
@@ -6026,13 +9042,12 @@
         <f>O3</f>
         <v/>
       </c>
-      <c r="P27">
-        <f>G27+H27+K27+L27+M27+N27+O27</f>
-        <v/>
+      <c r="P27" s="1" t="n">
+        <v>2095.6</v>
       </c>
       <c r="Q27" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6059,17 +9074,15 @@
         <f>E28*F28</f>
         <v/>
       </c>
-      <c r="H28">
-        <f>H27</f>
-        <v/>
+      <c r="H28" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I28">
         <f>I27</f>
         <v/>
       </c>
-      <c r="J28">
-        <f>J27</f>
-        <v/>
+      <c r="J28" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K28">
         <f>J28*I28</f>
@@ -6091,13 +9104,12 @@
         <f>O27</f>
         <v/>
       </c>
-      <c r="P28">
-        <f>G28+H28+K28+L28+M28+N28+O28</f>
-        <v/>
+      <c r="P28" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q28" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6124,17 +9136,15 @@
         <f>E29*F29</f>
         <v/>
       </c>
-      <c r="H29">
-        <f>H28</f>
-        <v/>
+      <c r="H29" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I29">
         <f>I28</f>
         <v/>
       </c>
-      <c r="J29">
-        <f>J28</f>
-        <v/>
+      <c r="J29" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K29">
         <f>J29*I29</f>
@@ -6156,13 +9166,12 @@
         <f>O28</f>
         <v/>
       </c>
-      <c r="P29">
-        <f>G29+H29+K29+L29+M29+N29+O29</f>
-        <v/>
+      <c r="P29" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q29" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6189,17 +9198,15 @@
         <f>E30*F30</f>
         <v/>
       </c>
-      <c r="H30">
-        <f>H29</f>
-        <v/>
+      <c r="H30" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I30">
         <f>I29</f>
         <v/>
       </c>
-      <c r="J30">
-        <f>J29</f>
-        <v/>
+      <c r="J30" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K30">
         <f>J30*I30</f>
@@ -6221,13 +9228,12 @@
         <f>O29</f>
         <v/>
       </c>
-      <c r="P30">
-        <f>G30+H30+K30+L30+M30+N30+O30</f>
-        <v/>
+      <c r="P30" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q30" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6254,17 +9260,15 @@
         <f>E31*F31</f>
         <v/>
       </c>
-      <c r="H31">
-        <f>H30</f>
-        <v/>
+      <c r="H31" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I31">
         <f>I30</f>
         <v/>
       </c>
-      <c r="J31">
-        <f>J30</f>
-        <v/>
+      <c r="J31" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K31">
         <f>J31*I31</f>
@@ -6286,13 +9290,12 @@
         <f>O30</f>
         <v/>
       </c>
-      <c r="P31">
-        <f>G31+H31+K31+L31+M31+N31+O31</f>
-        <v/>
+      <c r="P31" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q31" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6321,17 +9324,14 @@
       <c r="E32" t="n">
         <v>8</v>
       </c>
-      <c r="F32">
-        <f>F27</f>
-        <v/>
-      </c>
-      <c r="G32">
-        <f>E32*F32</f>
-        <v/>
-      </c>
-      <c r="H32">
-        <f>H5</f>
-        <v/>
+      <c r="F32" s="1" t="n">
+        <v>133.2</v>
+      </c>
+      <c r="G32" s="1" t="n">
+        <v>1065.6</v>
+      </c>
+      <c r="H32" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I32">
         <f>I5</f>
@@ -6360,13 +9360,12 @@
         <f>O5</f>
         <v/>
       </c>
-      <c r="P32">
-        <f>G32+H32+K32+L32+M32+N32+O32</f>
-        <v/>
+      <c r="P32" s="1" t="n">
+        <v>1935.6</v>
       </c>
       <c r="Q32" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6386,25 +9385,22 @@
         <f>E32</f>
         <v/>
       </c>
-      <c r="F33">
-        <f>F28</f>
-        <v/>
+      <c r="F33" s="1" t="n">
+        <v>147.2</v>
       </c>
       <c r="G33">
         <f>E33*F33</f>
         <v/>
       </c>
-      <c r="H33">
-        <f>H32</f>
-        <v/>
+      <c r="H33" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I33">
         <f>I32</f>
         <v/>
       </c>
-      <c r="J33">
-        <f>J32</f>
-        <v/>
+      <c r="J33" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K33">
         <f>J33*I33</f>
@@ -6426,13 +9422,12 @@
         <f>O32</f>
         <v/>
       </c>
-      <c r="P33">
-        <f>G33+H33+K33+L33+M33+N33+O33</f>
-        <v/>
+      <c r="P33" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q33" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6452,25 +9447,22 @@
         <f>E33</f>
         <v/>
       </c>
-      <c r="F34">
-        <f>F29</f>
-        <v/>
+      <c r="F34" s="1" t="n">
+        <v>133.2</v>
       </c>
       <c r="G34">
         <f>E34*F34</f>
         <v/>
       </c>
-      <c r="H34">
-        <f>H33</f>
-        <v/>
+      <c r="H34" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I34">
         <f>I33</f>
         <v/>
       </c>
-      <c r="J34">
-        <f>J33</f>
-        <v/>
+      <c r="J34" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K34">
         <f>J34*I34</f>
@@ -6492,13 +9484,12 @@
         <f>O33</f>
         <v/>
       </c>
-      <c r="P34">
-        <f>G34+H34+K34+L34+M34+N34+O34</f>
-        <v/>
+      <c r="P34" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q34" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6518,25 +9509,22 @@
         <f>E34</f>
         <v/>
       </c>
-      <c r="F35">
-        <f>F30</f>
-        <v/>
+      <c r="F35" s="1" t="n">
+        <v>147.2</v>
       </c>
       <c r="G35">
         <f>E35*F35</f>
         <v/>
       </c>
-      <c r="H35">
-        <f>H34</f>
-        <v/>
+      <c r="H35" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I35">
         <f>I34</f>
         <v/>
       </c>
-      <c r="J35">
-        <f>J34</f>
-        <v/>
+      <c r="J35" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K35">
         <f>J35*I35</f>
@@ -6558,13 +9546,12 @@
         <f>O34</f>
         <v/>
       </c>
-      <c r="P35">
-        <f>G35+H35+K35+L35+M35+N35+O35</f>
-        <v/>
+      <c r="P35" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q35" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6584,25 +9571,22 @@
         <f>E35</f>
         <v/>
       </c>
-      <c r="F36">
-        <f>F31</f>
-        <v/>
+      <c r="F36" s="1" t="n">
+        <v>133.2</v>
       </c>
       <c r="G36">
         <f>E36*F36</f>
         <v/>
       </c>
-      <c r="H36">
-        <f>H35</f>
-        <v/>
+      <c r="H36" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I36">
         <f>I35</f>
         <v/>
       </c>
-      <c r="J36">
-        <f>J35</f>
-        <v/>
+      <c r="J36" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K36">
         <f>J36*I36</f>
@@ -6624,13 +9608,12 @@
         <f>O35</f>
         <v/>
       </c>
-      <c r="P36">
-        <f>G36+H36+K36+L36+M36+N36+O36</f>
-        <v/>
+      <c r="P36" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q36" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6756,13 +9739,11 @@
       <c r="F39" s="1" t="n">
         <v>106.5</v>
       </c>
-      <c r="G39">
-        <f>E39*F39</f>
-        <v/>
-      </c>
-      <c r="H39">
-        <f>H3</f>
-        <v/>
+      <c r="G39" s="1" t="n">
+        <v>852</v>
+      </c>
+      <c r="H39" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I39">
         <f>I3</f>
@@ -6791,13 +9772,12 @@
         <f>O3</f>
         <v/>
       </c>
-      <c r="P39">
-        <f>G39+H39+K39+L39+M39+N39+O39</f>
-        <v/>
+      <c r="P39" s="1" t="n">
+        <v>1882</v>
       </c>
       <c r="Q39" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6824,17 +9804,15 @@
         <f>E40*F40</f>
         <v/>
       </c>
-      <c r="H40">
-        <f>H39</f>
-        <v/>
+      <c r="H40" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I40">
         <f>I39</f>
         <v/>
       </c>
-      <c r="J40">
-        <f>J39</f>
-        <v/>
+      <c r="J40" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K40">
         <f>J40*I40</f>
@@ -6856,13 +9834,12 @@
         <f>O39</f>
         <v/>
       </c>
-      <c r="P40">
-        <f>G40+H40+K40+L40+M40+N40+O40</f>
-        <v/>
+      <c r="P40" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q40" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6889,17 +9866,15 @@
         <f>E41*F41</f>
         <v/>
       </c>
-      <c r="H41">
-        <f>H40</f>
-        <v/>
+      <c r="H41" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I41">
         <f>I40</f>
         <v/>
       </c>
-      <c r="J41">
-        <f>J40</f>
-        <v/>
+      <c r="J41" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K41">
         <f>J41*I41</f>
@@ -6921,13 +9896,12 @@
         <f>O40</f>
         <v/>
       </c>
-      <c r="P41">
-        <f>G41+H41+K41+L41+M41+N41+O41</f>
-        <v/>
+      <c r="P41" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q41" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -6954,17 +9928,15 @@
         <f>E42*F42</f>
         <v/>
       </c>
-      <c r="H42">
-        <f>H41</f>
-        <v/>
+      <c r="H42" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I42">
         <f>I41</f>
         <v/>
       </c>
-      <c r="J42">
-        <f>J41</f>
-        <v/>
+      <c r="J42" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K42">
         <f>J42*I42</f>
@@ -6986,13 +9958,12 @@
         <f>O41</f>
         <v/>
       </c>
-      <c r="P42">
-        <f>G42+H42+K42+L42+M42+N42+O42</f>
-        <v/>
+      <c r="P42" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q42" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -7019,17 +9990,15 @@
         <f>E43*F43</f>
         <v/>
       </c>
-      <c r="H43">
-        <f>H42</f>
-        <v/>
+      <c r="H43" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I43">
         <f>I42</f>
         <v/>
       </c>
-      <c r="J43">
-        <f>J42</f>
-        <v/>
+      <c r="J43" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K43">
         <f>J43*I43</f>
@@ -7051,13 +10020,12 @@
         <f>O42</f>
         <v/>
       </c>
-      <c r="P43">
-        <f>G43+H43+K43+L43+M43+N43+O43</f>
-        <v/>
+      <c r="P43" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q43" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -7084,17 +10052,15 @@
         <f>E44*F44</f>
         <v/>
       </c>
-      <c r="H44">
-        <f>H42</f>
-        <v/>
+      <c r="H44" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="I44">
         <f>I42</f>
         <v/>
       </c>
-      <c r="J44">
-        <f>J42</f>
-        <v/>
+      <c r="J44" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K44">
         <f>J44*I44</f>
@@ -7116,13 +10082,12 @@
         <f>O42</f>
         <v/>
       </c>
-      <c r="P44">
-        <f>G44+H44+K44+L44+M44+N44+O44</f>
-        <v/>
+      <c r="P44" s="1" t="n">
+        <v>1030</v>
       </c>
       <c r="Q44" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -7151,17 +10116,14 @@
       <c r="E45" t="n">
         <v>8</v>
       </c>
-      <c r="F45">
-        <f>F39</f>
-        <v/>
-      </c>
-      <c r="G45">
-        <f>E45*F45</f>
-        <v/>
-      </c>
-      <c r="H45">
-        <f>H5</f>
-        <v/>
+      <c r="F45" s="1" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="G45" s="1" t="n">
+        <v>852</v>
+      </c>
+      <c r="H45" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I45">
         <f>I5</f>
@@ -7190,13 +10152,12 @@
         <f>O5</f>
         <v/>
       </c>
-      <c r="P45">
-        <f>G45+H45+K45+L45+M45+N45+O45</f>
-        <v/>
+      <c r="P45" s="1" t="n">
+        <v>1722</v>
       </c>
       <c r="Q45" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -7216,25 +10177,22 @@
         <f>E45</f>
         <v/>
       </c>
-      <c r="F46">
-        <f>F40</f>
-        <v/>
+      <c r="F46" s="1" t="n">
+        <v>120.5</v>
       </c>
       <c r="G46">
         <f>E46*F46</f>
         <v/>
       </c>
-      <c r="H46">
-        <f>H45</f>
-        <v/>
+      <c r="H46" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I46">
         <f>I45</f>
         <v/>
       </c>
-      <c r="J46">
-        <f>J45</f>
-        <v/>
+      <c r="J46" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K46">
         <f>J46*I46</f>
@@ -7256,13 +10214,12 @@
         <f>O45</f>
         <v/>
       </c>
-      <c r="P46">
-        <f>G46+H46+K46+L46+M46+N46+O46</f>
-        <v/>
+      <c r="P46" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q46" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -7282,25 +10239,22 @@
         <f>E46</f>
         <v/>
       </c>
-      <c r="F47">
-        <f>F41</f>
-        <v/>
+      <c r="F47" s="1" t="n">
+        <v>106.5</v>
       </c>
       <c r="G47">
         <f>E47*F47</f>
         <v/>
       </c>
-      <c r="H47">
-        <f>H46</f>
-        <v/>
+      <c r="H47" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I47">
         <f>I46</f>
         <v/>
       </c>
-      <c r="J47">
-        <f>J46</f>
-        <v/>
+      <c r="J47" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K47">
         <f>J47*I47</f>
@@ -7322,13 +10276,12 @@
         <f>O46</f>
         <v/>
       </c>
-      <c r="P47">
-        <f>G47+H47+K47+L47+M47+N47+O47</f>
-        <v/>
+      <c r="P47" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q47" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -7348,25 +10301,22 @@
         <f>E47</f>
         <v/>
       </c>
-      <c r="F48">
-        <f>F42</f>
-        <v/>
+      <c r="F48" s="1" t="n">
+        <v>120.5</v>
       </c>
       <c r="G48">
         <f>E48*F48</f>
         <v/>
       </c>
-      <c r="H48">
-        <f>H47</f>
-        <v/>
+      <c r="H48" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I48">
         <f>I47</f>
         <v/>
       </c>
-      <c r="J48">
-        <f>J47</f>
-        <v/>
+      <c r="J48" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K48">
         <f>J48*I48</f>
@@ -7388,13 +10338,12 @@
         <f>O47</f>
         <v/>
       </c>
-      <c r="P48">
-        <f>G48+H48+K48+L48+M48+N48+O48</f>
-        <v/>
+      <c r="P48" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q48" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -7414,25 +10363,22 @@
         <f>E48</f>
         <v/>
       </c>
-      <c r="F49">
-        <f>F43</f>
-        <v/>
+      <c r="F49" s="1" t="n">
+        <v>106.5</v>
       </c>
       <c r="G49">
         <f>E49*F49</f>
         <v/>
       </c>
-      <c r="H49">
-        <f>H48</f>
-        <v/>
+      <c r="H49" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I49">
         <f>I48</f>
         <v/>
       </c>
-      <c r="J49">
-        <f>J48</f>
-        <v/>
+      <c r="J49" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K49">
         <f>J49*I49</f>
@@ -7454,13 +10400,12 @@
         <f>O48</f>
         <v/>
       </c>
-      <c r="P49">
-        <f>G49+H49+K49+L49+M49+N49+O49</f>
-        <v/>
+      <c r="P49" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q49" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>
@@ -7480,25 +10425,22 @@
         <f>E48</f>
         <v/>
       </c>
-      <c r="F50">
-        <f>F44</f>
-        <v/>
+      <c r="F50" s="1" t="n">
+        <v>120.5</v>
       </c>
       <c r="G50">
         <f>E50*F50</f>
         <v/>
       </c>
-      <c r="H50">
-        <f>H48</f>
-        <v/>
+      <c r="H50" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="I50">
         <f>I48</f>
         <v/>
       </c>
-      <c r="J50">
-        <f>J48</f>
-        <v/>
+      <c r="J50" s="1" t="n">
+        <v>72</v>
       </c>
       <c r="K50">
         <f>J50*I50</f>
@@ -7520,13 +10462,12 @@
         <f>O48</f>
         <v/>
       </c>
-      <c r="P50">
-        <f>G50+H50+K50+L50+M50+N50+O50</f>
-        <v/>
+      <c r="P50" s="1" t="n">
+        <v>870</v>
       </c>
       <c r="Q50" s="1" t="inlineStr">
         <is>
-          <t>大件单价见规格单价表；演示价·大件示意</t>
+          <t>模组单价见规格单价表；箱体/电源见本册价目；演示价·收口示意（电源只数为演示维护值）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add control-box pricing, quote totals, and clearer tender-agnostic skills.
Migrate the control cabinet BOM into the accounting book, require three-tier quote totals, pin pitch/steel/hoop rules, ask questions with suggested options, and sync confirmation docs plus the fill guide.
</commit_message>
<xml_diff>
--- a/chuangdi/数据/核算口径表-演示.xlsx
+++ b/chuangdi/数据/核算口径表-演示.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="电源" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="支架" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安装抱箍和螺钉" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每平米收口" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="控制箱" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每平米收口" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,14 +452,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>本文件整理自大模组核算原表：辅材 BOM、每平米收口结构、箱体/电源/支架/抱箍价目。「每平米收口」样例行是历史底稿，项目报价由 Agent 按招标+规格+本表规则重算本项目收口，不是样例×面积。</t>
+          <t>本文件整理自大模组核算原表：辅材 BOM、每平米收口结构、箱体/电源/支架/抱箍/控制箱价目。「每平米收口」样例行是历史底稿，项目报价由 Agent 按招标+规格+本表规则重算本项目收口，不是样例×面积。</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>三件套：规格单价表（模组/灯珠/套件及物理箱 SKU）+ 本表（BOM、收口结构、元/㎡箱体与电源/支架/抱箍价目）+ 计价 skill。详见方案/场景演示建议口径.md、原表公式与经验配量确认.md。</t>
+          <t>三件套：规格单价表（模组/灯珠/套件及物理箱 SKU）+ 本表（BOM、收口结构、元/㎡箱体与电源/支架/抱箍/控制箱价目）+ 计价 skill。详见方案/场景演示建议口径.md、原表公式与经验配量确认.md。</t>
         </is>
       </c>
     </row>
@@ -479,14 +480,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>价目页「箱体」「电源」「支架」「安装抱箍和螺钉」自原表迁入；正式稿单价空/0 由成本维护。规格单价表「箱体单价」仅作物料核对，平方单价中的箱体元/㎡以本册「箱体」为准。</t>
+          <t>价目页「箱体」「电源」「支架」「安装抱箍和螺钉」「控制箱」自原表迁入；正式稿单价空/0 由成本维护。规格单价表「箱体单价」仅作物料核对，平方单价中的箱体元/㎡以本册「箱体」为准。报价单「控制系统」取本册「控制箱」汇总（每套），形态加价见报价单 skill。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>不转入屏体清单样例页、压铸铝控制箱。招标用抄录面积。供应商名不转入。</t>
+          <t>不转入屏体清单样例页。招标用抄录面积。供应商名不转入。</t>
         </is>
       </c>
     </row>
@@ -500,7 +501,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>【演示副本】辅材 BOM、箱体/电源/支架/抱箍价目已填模拟单价（黄底）并滚出可读汇总。「常规电源数量」等为演示维护示意，供 POC 重算本项目收口；不是未确认的正式成本定额。本文件不是创迪采购价。正式稿单价由成本维护；项目报价按招标+规格重算，非样例×面积。</t>
+          <t>【演示副本】辅材 BOM、箱体/电源/支架/抱箍/控制箱价目已填模拟单价（黄底）并滚出可读汇总。「常规电源数量」等为演示维护示意，供 POC 重算本项目收口；不是未确认的正式成本定额。本文件不是创迪采购价。正式稿单价由成本维护；项目报价按招标+规格重算，非样例×面积。</t>
         </is>
       </c>
     </row>
@@ -2958,10 +2959,10 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>1.5</v>
+        <v>420</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>1.5</v>
+        <v>420</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
@@ -3016,10 +3017,10 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>1.5</v>
+        <v>95</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>1.5</v>
+        <v>95</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
@@ -3045,10 +3046,10 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>1.5</v>
+        <v>45</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>30</v>
+        <v>900</v>
       </c>
       <c r="F22" t="n">
         <v>20</v>
@@ -3074,10 +3075,10 @@
         </is>
       </c>
       <c r="D23" s="1" t="n">
-        <v>1.5</v>
+        <v>28</v>
       </c>
       <c r="E23" s="1" t="n">
-        <v>1.5</v>
+        <v>28</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
@@ -3103,10 +3104,10 @@
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>1.5</v>
+        <v>85</v>
       </c>
       <c r="E24" s="1" t="n">
-        <v>1.5</v>
+        <v>85</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
@@ -3132,10 +3133,10 @@
         </is>
       </c>
       <c r="D25" s="1" t="n">
-        <v>1.5</v>
+        <v>85</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>1.5</v>
+        <v>85</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
@@ -3219,10 +3220,10 @@
         </is>
       </c>
       <c r="D28" s="1" t="n">
-        <v>1.5</v>
+        <v>28</v>
       </c>
       <c r="E28" s="1" t="n">
-        <v>0.45</v>
+        <v>8.4</v>
       </c>
       <c r="F28" t="n">
         <v>0.3</v>
@@ -4045,7 +4046,7 @@
     </row>
     <row r="57">
       <c r="E57" s="1" t="n">
-        <v>2866.985</v>
+        <v>4450.435</v>
       </c>
     </row>
     <row r="58">
@@ -4055,7 +4056,7 @@
         </is>
       </c>
       <c r="E58" s="1" t="n">
-        <v>286.6985</v>
+        <v>445.0435</v>
       </c>
     </row>
     <row r="59"/>
@@ -7472,6 +7473,1362 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>BOM层级</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>子项物料编码</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>物料名称</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>含税单价</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3000001386</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>可变信息标志控制箱（单相含控制卡--无信号防雷版）/KXB-10P-A1-KZX+KZ03/400*610*140/SGCC=1.2 户外7035</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>680</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>680</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>..2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2300001283</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>可变信息标志控制箱（单相含控制卡-无信号防雷版）/KXB-10P-A1-KZX+KZ03/400*610*140/SGCC=1.2 户外7035 裸机</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>680</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>680</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2200000649</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>服务区情报板单相控制箱（背抱安装）箱体/KXB-KZ03D-D1/400*610*140/SGCC=1.2 户外7035</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>680</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>680</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1000000932</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>多媒体播放盒/GX30T</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>420</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>420</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1500000042</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>开关电源/LM25-23B05/5V/5A 25W/效率88%/工作温度范围：-30℃to +70℃/VEN00112</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1700000010</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>单相电源防雷器/CD-D/AC20-2（丝印创迪LOGO）/VEN00054</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>85</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>85</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1900000039</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>光探头/ALP050-1.5M-P/CON4-2.54插头</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1000000515</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>空开/DZ47SC63(63A,1P)/N</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1000000464</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>空开/DZ47sN1C32(32A,1P)/N</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>84</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1300000116</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AC30模数化插座/250V/10-16A/3孔</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1600000102</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>过线圈/PG29/尼龙/白色</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1000000480</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>空开背条/L=1000*35*7.5mm/C45导轨，1mm厚，国标</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1300000120</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>接线端子固定卡/E-UK</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1300000153</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>10孔桥型接线排/8*12地排/110.8*31.8*12.5mm/绿色</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1300000154</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>10孔桥型接线排/8*12零排/110.8*31.8*12.5mm/蓝色</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1600000063</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>3合1螺钉/M4*8/碳钢/镀白锌</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1600000027</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>圆头十字螺钉/M4*8/碳钢/镀白锌</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1600000064</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>3合1螺钉/M4×16/碳钢/镀白锌</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1600000100</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>3合1螺钉/M3*6/碳钢/包黑色</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1600000004</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>螺母/M6/碳钢/镀白锌</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1600000043</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>不锈钢弹垫/M6/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1600000049</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>不锈钢平垫/M6/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1400000142</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>一拖一5V单元板电源线/主线长0.5m 分支线长0.3m  接线叉SNB2-4 /分支线BVR铜软0.75mm² 主线国标BVR铜软2.5mm²</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1700003108</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RJ45网口防尘塞/硅胶 黑色</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1400000060</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘阻燃软电线/ZR BVR1*1.5mm²电压450-750V/红色</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1400000059</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘阻燃软电线/ZR BVR1*1.5mm²电压450-750V/黑色</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1400000061</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘阻燃软电线/ZR BVR1*1.5mm²电压450-750V/黄绿色</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1400000063</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘阻燃软电线/ZR BVR1*1.5mm²电压450-750V/蓝色</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1400000065</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘阻燃软电线/ZR BVR1*1.5mm²电压450-750V/棕色</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1400000056</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘软电缆/BVR1*2.5mm²电压450-750V/蓝色</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1400000058</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘软电缆/BVR1*2.5mm²电压450-750V/棕色</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1400000054</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘软电缆/BVR1*2.5mm²电压450-750V/黄绿色</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1400000093</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>铜芯聚氯乙烯绝缘软电缆/BVR1*4mm²电压450-750V/棕色</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1300000129</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>冷压接线端子/SNB2-3/国标紫铜U型/16*5.7*0.8mm</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="F35" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1300000126</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>冷压接线端子/C45-2.5/插片形DZ47国标紫铜/13*4.8*0.7mm</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="F36" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1300000151</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>冷压接线端子/C45-6/插片形DZ47国标紫铜/13*4.8*0.7mm</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="F37" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1300000128</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>冷压接线端子/RNB2-6/国标紫铜O型/21.7*12*0.8mm</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1300000127</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>冷压接线端子/RNB2-4/国标紫铜O型/14.4*6.6*0.8mm</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F39" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1700002806</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>尼龙扎带/3*150mm/黑色</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F40" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1800000465</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>重庆创迪LOGO图样/CD-LG-CDKJ</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1800000005</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>亚银标签纸/50*125</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1800000012</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>合格证不干胶贴/φ25</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1800000967</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>可变信息标志控制箱单相含控制卡-无信号防雷版使用说明书</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E44" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1800000968</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>可变信息标志单相洞外控制箱产品无信号防雷版接线示意图/150 *210 /A4光面黄底不干胶标签贴纸</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>...3</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1800000109</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>纸箱/CDTPJ-ZXL-D17/内670*410*150外685*425*165/ 5层瓦楞 本色</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>..2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1700000384</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>控制箱背抱 几字连接板/KXB-KZ03-A5/140*40*33/SGCC=3 户外7035</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="E47" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>..2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1600000036</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>外六角螺栓/M10*30/不锈钢/本色</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E48" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F48" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>..2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1600000044</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>不锈钢弹垫/M10/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E49" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F49" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>..2</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1600000050</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>不锈钢平垫/M10/不锈钢 A2-70/本色</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F50" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>.1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1700003261</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>PA尼龙波纹管（闭口）/AD34.5内径29mm外径34.5mm PA6尼龙/工作温度-40℃-100℃/黑色</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="E51" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="F51" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>总计辅材和箱体10平方（演示汇总）</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="n">
+        <v>3018.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Q50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -7736,10 +9093,10 @@
         <v>16</v>
       </c>
       <c r="O5" s="1" t="n">
-        <v>306.6985</v>
+        <v>465.0435</v>
       </c>
       <c r="P5" s="1" t="n">
-        <v>2931.34</v>
+        <v>3089.68</v>
       </c>
       <c r="Q5" s="1" t="inlineStr">
         <is>

</xml_diff>